<commit_message>
test(oracle): cover structured defined names
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/excel-oracle/calamine-native-tables/fixture.xlsx
+++ b/tests/excel-oracle/calamine-native-tables/fixture.xlsx
@@ -3,13 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71032ADA-9D54-4190-B322-C7475714B755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2224F4EB-1D43-40A6-A97F-3AB9BD32F08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{48B4A326-FF7C-4C73-B43F-61F943088170}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{927B3E41-5D21-4B84-8F56-CF76DA281286}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Other" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="CoercedAmounts">VALUE(SalesTable[Amount])</definedName>
+    <definedName name="LocalAmounts" localSheetId="0">SalesTable[Amount]</definedName>
+    <definedName name="SalesAllAmounts">SalesTable[[#All],[Amount]]</definedName>
+    <definedName name="SalesAmounts">SalesTable[Amount]</definedName>
+    <definedName name="ScopeProbe" localSheetId="0">Data!$B$3</definedName>
+    <definedName name="ScopeProbe">Data!$B$2</definedName>
+  </definedNames>
   <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -31,6 +40,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -104,11 +135,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AB97B46-BF6D-4E74-9E1D-0AE3C2BEA7D3}" name="SalesTable" displayName="SalesTable" ref="A1:B4" totalsRowShown="0">
-  <autoFilter ref="A1:B4" xr:uid="{1AB97B46-BF6D-4E74-9E1D-0AE3C2BEA7D3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6E5306B5-3344-4256-B09E-314D5F9C7211}" name="SalesTable" displayName="SalesTable" ref="A1:B4" totalsRowShown="0">
+  <autoFilter ref="A1:B4" xr:uid="{6E5306B5-3344-4256-B09E-314D5F9C7211}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{143BA369-A0C7-407D-A85F-C822F524E944}" name="Key"/>
-    <tableColumn id="2" xr3:uid="{7FE1DFBE-EE98-4593-81AE-02851A33374C}" name="Amount"/>
+    <tableColumn id="1" xr3:uid="{FF44DDAE-8CA8-418A-AA9E-67B66F216B11}" name="Key"/>
+    <tableColumn id="2" xr3:uid="{56B50E25-F9EA-4B30-86FD-3A9EA1A2010A}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -430,8 +461,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB6D6EE9-CCC5-4EC6-AD10-D546C0920A8B}">
-  <dimension ref="A1:D4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07955DB1-AB91-4805-BB1A-6705FBE582B8}">
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.36328125" customWidth="1"/>
@@ -464,6 +495,10 @@
       <c r="B3">
         <v>20</v>
       </c>
+      <c r="D3">
+        <f>SUM(SalesAmounts)</f>
+        <v>60</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -471,6 +506,46 @@
       </c>
       <c r="B4">
         <v>30</v>
+      </c>
+      <c r="D4">
+        <f>SUM(LocalAmounts)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <f>SUM(SalesAllAmounts)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <f>SUM(CoercedAmounts)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D7" t="e" cm="1">
+        <f t="array" ref="D7">SUM(VALUE(SalesAllAmounts))</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D8" cm="1">
+        <f t="array" ref="D8">MATCH(20,VALUE(SalesAllAmounts),1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D9" cm="1">
+        <f t="array" ref="D9">MATCH(20,VALUE(SalesAllAmounts),0)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <f>ScopeProbe</f>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -479,4 +554,20 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8B83F7-66E3-4E04-B388-86F23471AB0C}">
+  <dimension ref="D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <f>ScopeProbe</f>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(eval): allow forward defined-name dependencies
Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/excel-oracle/calamine-native-tables/fixture.xlsx
+++ b/tests/excel-oracle/calamine-native-tables/fixture.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2224F4EB-1D43-40A6-A97F-3AB9BD32F08B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A2A188B-57BE-4590-9203-52EBE457E79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{927B3E41-5D21-4B84-8F56-CF76DA281286}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{A47C26D4-ED16-403F-81B6-6CB3159107C2}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -13,6 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="CoercedAmounts">VALUE(SalesTable[Amount])</definedName>
+    <definedName name="DerivedAmounts">SUM(SalesAmounts)</definedName>
     <definedName name="LocalAmounts" localSheetId="0">SalesTable[Amount]</definedName>
     <definedName name="SalesAllAmounts">SalesTable[[#All],[Amount]]</definedName>
     <definedName name="SalesAmounts">SalesTable[Amount]</definedName>
@@ -135,11 +136,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6E5306B5-3344-4256-B09E-314D5F9C7211}" name="SalesTable" displayName="SalesTable" ref="A1:B4" totalsRowShown="0">
-  <autoFilter ref="A1:B4" xr:uid="{6E5306B5-3344-4256-B09E-314D5F9C7211}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD35DBC9-0396-45AD-856D-7EB53054F1F2}" name="SalesTable" displayName="SalesTable" ref="A1:B4" totalsRowShown="0">
+  <autoFilter ref="A1:B4" xr:uid="{CD35DBC9-0396-45AD-856D-7EB53054F1F2}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{FF44DDAE-8CA8-418A-AA9E-67B66F216B11}" name="Key"/>
-    <tableColumn id="2" xr3:uid="{56B50E25-F9EA-4B30-86FD-3A9EA1A2010A}" name="Amount"/>
+    <tableColumn id="1" xr3:uid="{79ACDF2E-5BF9-4A2E-9668-632D2B7B4326}" name="Key"/>
+    <tableColumn id="2" xr3:uid="{526D47E1-CCAC-4370-8C00-8CC137BDE499}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -461,8 +462,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07955DB1-AB91-4805-BB1A-6705FBE582B8}">
-  <dimension ref="A1:D10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{421CCBA8-F2FE-4480-B905-8A6209286C4A}">
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.36328125" customWidth="1"/>
@@ -548,6 +549,12 @@
         <v>20</v>
       </c>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <f>DerivedAmounts</f>
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -557,7 +564,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E8B83F7-66E3-4E04-B388-86F23471AB0C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7655AF0C-8230-4E86-8531-728D200FDF8F}">
   <dimension ref="D2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>

</xml_diff>